<commit_message>
added all data field selections
</commit_message>
<xml_diff>
--- a/outputs/galicia_precip_monthly_1997_2026_v2.xlsx
+++ b/outputs/galicia_precip_monthly_1997_2026_v2.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Documents\ss_ML_local\galicia-climate-analysis\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE701C89-9035-4A43-A359-3B0299C785A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12C106C-0B21-422E-AB8B-9D9DAF62A958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2415" yWindow="375" windowWidth="25995" windowHeight="14955" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2415" yWindow="375" windowWidth="25995" windowHeight="14955" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="station_month_matrix" sheetId="1" r:id="rId1"/>
-    <sheet name="wide" sheetId="2" r:id="rId2"/>
-    <sheet name="long" sheetId="3" r:id="rId3"/>
+    <sheet name="graph" sheetId="4" r:id="rId2"/>
+    <sheet name="wide" sheetId="2" r:id="rId3"/>
+    <sheet name="long" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
@@ -563,6 +564,55 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>219956</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>877</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4FB96C3D-C788-06F1-F13E-0318DDF534D4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6315956" cy="6287377"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -13344,6 +13394,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87FDA264-3626-4852-ACE5-7B103DA402A5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:S268"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -28025,10 +28085,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E3472"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="12" max="12" width="9.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>